<commit_message>
feat(examples): synthetic 846/812/867 sets with planted defects and tests
The defective 812 carries the classic backwards-keyed credit signature
(total gap = twice the mis-signed amount); the 846 plants a mystery ZZ
quantity bucket and a missing committed bucket (NOT TESTED, not a false
fail); the 867 lies in both its header total and CTT. Streamlit gains
six scenarios; README coverage table updated.
</commit_message>
<xml_diff>
--- a/examples/specs/810_reference_spec.xlsx
+++ b/examples/specs/810_reference_spec.xlsx
@@ -1497,7 +1497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1530,243 +1530,264 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  (blank)   header/summary area, first occurrence</t>
+          <t xml:space="preserve">                  (blank)      header/summary area, first occurrence</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  PO1       each occurrence of the PO1 loop (per-line rule;</t>
+          <t xml:space="preserve">                  PO1          each occurrence of the PO1 loop (per-line</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                            target must use lines[] notation)</t>
+          <t xml:space="preserve">                               rule; target must use lines[] notation)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  N1[ST]    the N1 loop whose N101 = ST</t>
+          <t xml:space="preserve">                  N1[ST]       the N1 loop whose N101 = ST</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                  REF[DP]   the REF segment whose REF01 = DP</t>
+          <t xml:space="preserve">                  REF[DP]      the REF segment whose REF01 = DP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                The [qualifier] always matches element 01 of that segment.</t>
+          <t xml:space="preserve">                  LIN&gt;QTY[QA]  per-line on the LIN loop, but the source</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>TARGET FIELD    Dot path into the output: order.po_number, ship_to.name,</t>
+          <t xml:space="preserve">                               field reads the QTY whose QTY01 = QA (for</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                lines[].qty, summary.line_count.</t>
+          <t xml:space="preserve">                               repeating qualified segments in a loop)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>RULE TYPE       DIRECT       source value lands in target (after type/format</t>
+          <t xml:space="preserve">                The [qualifier] always matches element 01 of that segment.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                             conversion)</t>
+          <t>TARGET FIELD    Dot path into the output: order.po_number, ship_to.name,</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                CONDITIONAL  Condition (Coded) decides between Then and Else</t>
+          <t xml:space="preserve">                lines[].qty, summary.line_count.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                CODE_LIST    source value translated via the named code list</t>
+          <t>RULE TYPE       DIRECT       source value lands in target (after type/format</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                CONSTANT     hardcoded value from Default Value (no source)</t>
+          <t xml:space="preserve">                             conversion)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                LOOP_COUNT   target = occurrence count of the loop named in</t>
+          <t xml:space="preserve">                CONDITIONAL  Condition (Coded) decides between Then and Else</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                             Source Field (e.g. PO1)</t>
+          <t xml:space="preserve">                CODE_LIST    source value translated via the named code list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>CONDITION       (Text) is documentation for humans. (Coded) is what the</t>
+          <t xml:space="preserve">                CONSTANT     hardcoded value from Default Value (no source)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                engine runs:  N101 = 'ST'</t>
+          <t xml:space="preserve">                LOOP_COUNT   target = occurrence count of the loop named in</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                              BEG02 != 'SA'</t>
+          <t xml:space="preserve">                             Source Field (e.g. PO1)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                              PO103 IN ('EA', 'CA')</t>
+          <t>CONDITION       (Text) is documentation for humans. (Coded) is what the</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                              EXISTS(REF02)</t>
+          <t xml:space="preserve">                engine runs:  N101 = 'ST'</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Join with AND. Values always in single quotes.</t>
+          <t xml:space="preserve">                              BEG02 != 'SA'</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>THEN / ELSE     SOURCE (map the source value), SKIP (field must be absent),</t>
+          <t xml:space="preserve">                              PO103 IN ('EA', 'CA')</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                BLANK (present but empty), or a 'quoted literal'.</t>
+          <t xml:space="preserve">                              EXISTS(REF02)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Else defaults to SKIP when left empty.</t>
+          <t xml:space="preserve">                Join with AND. Values always in single quotes.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>DEFAULT VALUE   CONSTANT rules: the hardcoded value. Other rules: fallback</t>
+          <t>THEN / ELSE     SOURCE (map the source value), SKIP (field must be absent),</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                used when the source element is empty/absent.</t>
+          <t xml:space="preserve">                BLANK (present but empty), or a 'quoted literal'.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>DATA TYPE       string | integer | decimal | date | time</t>
+          <t xml:space="preserve">                Else defaults to SKIP when left empty.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>FORMAT          date:    strftime pattern of the OUTPUT value, e.g. %Y-%m-%d</t>
+          <t>DEFAULT VALUE   CONSTANT rules: the hardcoded value. Other rules: fallback</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                         (X12 source dates are read as CCYYMMDD/YYMMDD)</t>
+          <t xml:space="preserve">                used when the source element is empty/absent.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                decimal: places:2 (output has 2 decimal places) and/or</t>
+          <t>DATA TYPE       string | integer | decimal | date | time</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                         implied:2 (source is X12 N2 — implied 2 decimals)</t>
+          <t>FORMAT          date:    strftime pattern of the OUTPUT value, e.g. %Y-%m-%d</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                string:  len:1..30 (allowed output length range)</t>
+          <t xml:space="preserve">                         (X12 source dates are read as CCYYMMDD/YYMMDD)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">                Combine with ; e.g.  implied:2;places:2</t>
+          <t xml:space="preserve">                decimal: places:2 (output has 2 decimal places) and/or</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>CODE LISTS      Long format on the CodeLists sheet; Code List Ref names the</t>
+          <t xml:space="preserve">                         implied:2 (source is X12 N2 — implied 2 decimals)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                string:  len:1..30 (allowed output length range)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                Combine with ; e.g.  implied:2;places:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>CODE LISTS      Long format on the CodeLists sheet; Code List Ref names the</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">                List Name value.</t>
         </is>

</xml_diff>